<commit_message>
fixing dataframe dtype for gh actions
</commit_message>
<xml_diff>
--- a/helpers/testing/test_output.xlsx
+++ b/helpers/testing/test_output.xlsx
@@ -964,9 +964,11 @@
       <c r="AJ4" s="3" t="n"/>
       <c r="AK4" s="3" t="n"/>
       <c r="AL4" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM4" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM4" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN4" s="3" t="n"/>
     </row>
     <row r="5">
@@ -1058,9 +1060,11 @@
       <c r="AJ5" s="3" t="n"/>
       <c r="AK5" s="3" t="n"/>
       <c r="AL5" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM5" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM5" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN5" s="3" t="n"/>
     </row>
     <row r="6">
@@ -1152,11 +1156,9 @@
       <c r="AJ6" s="3" t="n"/>
       <c r="AK6" s="3" t="n"/>
       <c r="AL6" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM6" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM6" s="10" t="n"/>
       <c r="AN6" s="3" t="n"/>
     </row>
     <row r="7">
@@ -1436,11 +1438,9 @@
       <c r="AJ9" s="3" t="n"/>
       <c r="AK9" s="3" t="n"/>
       <c r="AL9" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM9" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM9" s="10" t="n"/>
       <c r="AN9" s="3" t="n"/>
     </row>
     <row r="10">
@@ -1532,11 +1532,9 @@
       <c r="AJ10" s="3" t="n"/>
       <c r="AK10" s="3" t="n"/>
       <c r="AL10" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM10" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM10" s="10" t="n"/>
       <c r="AN10" s="3" t="n"/>
     </row>
     <row r="11">
@@ -1631,7 +1629,7 @@
         <v>1</v>
       </c>
       <c r="AM11" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN11" s="3" t="n"/>
     </row>
@@ -1724,9 +1722,11 @@
       <c r="AJ12" s="3" t="n"/>
       <c r="AK12" s="3" t="n"/>
       <c r="AL12" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM12" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM12" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN12" s="3" t="n"/>
     </row>
     <row r="13">
@@ -1821,7 +1821,7 @@
         <v>1</v>
       </c>
       <c r="AM13" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN13" s="3" t="n"/>
     </row>
@@ -1917,7 +1917,7 @@
         <v>1</v>
       </c>
       <c r="AM14" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN14" s="3" t="n"/>
     </row>
@@ -2010,11 +2010,9 @@
       <c r="AJ15" s="3" t="n"/>
       <c r="AK15" s="3" t="n"/>
       <c r="AL15" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM15" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM15" s="10" t="n"/>
       <c r="AN15" s="3" t="n"/>
     </row>
     <row r="16">
@@ -2109,7 +2107,7 @@
         <v>1</v>
       </c>
       <c r="AM16" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN16" s="3" t="n"/>
     </row>
@@ -2202,11 +2200,9 @@
       <c r="AJ17" s="3" t="n"/>
       <c r="AK17" s="3" t="n"/>
       <c r="AL17" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM17" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM17" s="10" t="n"/>
       <c r="AN17" s="3" t="n"/>
     </row>
     <row r="18">
@@ -2301,7 +2297,7 @@
         <v>1</v>
       </c>
       <c r="AM18" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN18" s="3" t="n"/>
     </row>
@@ -2394,9 +2390,11 @@
       <c r="AJ19" s="3" t="n"/>
       <c r="AK19" s="3" t="n"/>
       <c r="AL19" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM19" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM19" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN19" s="3" t="n"/>
     </row>
     <row r="20">
@@ -2488,11 +2486,9 @@
       <c r="AJ20" s="3" t="n"/>
       <c r="AK20" s="3" t="n"/>
       <c r="AL20" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM20" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM20" s="10" t="n"/>
       <c r="AN20" s="3" t="n"/>
     </row>
     <row r="21">
@@ -2681,7 +2677,7 @@
         <v>1</v>
       </c>
       <c r="AM22" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN22" s="3" t="n"/>
     </row>
@@ -2774,11 +2770,9 @@
       <c r="AJ23" s="3" t="n"/>
       <c r="AK23" s="3" t="n"/>
       <c r="AL23" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM23" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM23" s="10" t="n"/>
       <c r="AN23" s="3" t="n"/>
     </row>
     <row r="24">
@@ -2873,7 +2867,7 @@
         <v>1</v>
       </c>
       <c r="AM24" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN24" s="3" t="n"/>
     </row>
@@ -2969,7 +2963,7 @@
         <v>1</v>
       </c>
       <c r="AM25" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN25" s="3" t="n"/>
     </row>
@@ -3250,11 +3244,9 @@
       <c r="AJ28" s="3" t="n"/>
       <c r="AK28" s="3" t="n"/>
       <c r="AL28" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM28" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM28" s="10" t="n"/>
       <c r="AN28" s="3" t="n"/>
     </row>
     <row r="29">
@@ -3346,9 +3338,11 @@
       <c r="AJ29" s="3" t="n"/>
       <c r="AK29" s="3" t="n"/>
       <c r="AL29" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM29" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM29" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN29" s="3" t="n"/>
     </row>
     <row r="30">
@@ -3537,7 +3531,7 @@
         <v>1</v>
       </c>
       <c r="AM31" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN31" s="3" t="n"/>
     </row>
@@ -3633,7 +3627,7 @@
         <v>1</v>
       </c>
       <c r="AM32" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN32" s="3" t="n"/>
     </row>
@@ -3729,7 +3723,7 @@
         <v>1</v>
       </c>
       <c r="AM33" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN33" s="3" t="n"/>
     </row>
@@ -3916,9 +3910,11 @@
       <c r="AJ35" s="3" t="n"/>
       <c r="AK35" s="3" t="n"/>
       <c r="AL35" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM35" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM35" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN35" s="3" t="n"/>
     </row>
     <row r="36">
@@ -4010,11 +4006,9 @@
       <c r="AJ36" s="3" t="n"/>
       <c r="AK36" s="3" t="n"/>
       <c r="AL36" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM36" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM36" s="10" t="n"/>
       <c r="AN36" s="3" t="n"/>
     </row>
     <row r="37">
@@ -4109,7 +4103,7 @@
         <v>1</v>
       </c>
       <c r="AM37" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN37" s="3" t="n"/>
     </row>
@@ -4202,11 +4196,9 @@
       <c r="AJ38" s="3" t="n"/>
       <c r="AK38" s="3" t="n"/>
       <c r="AL38" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM38" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM38" s="10" t="n"/>
       <c r="AN38" s="3" t="n"/>
     </row>
     <row r="39">
@@ -4392,9 +4384,11 @@
       <c r="AJ40" s="3" t="n"/>
       <c r="AK40" s="3" t="n"/>
       <c r="AL40" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM40" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM40" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN40" s="3" t="n"/>
     </row>
     <row r="41">
@@ -4489,7 +4483,7 @@
         <v>1</v>
       </c>
       <c r="AM41" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN41" s="3" t="n"/>
     </row>
@@ -4585,7 +4579,7 @@
         <v>1</v>
       </c>
       <c r="AM42" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN42" s="3" t="n"/>
     </row>
@@ -4678,11 +4672,9 @@
       <c r="AJ43" s="3" t="n"/>
       <c r="AK43" s="3" t="n"/>
       <c r="AL43" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM43" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM43" s="10" t="n"/>
       <c r="AN43" s="3" t="n"/>
     </row>
     <row r="44">
@@ -4871,7 +4863,7 @@
         <v>1</v>
       </c>
       <c r="AM45" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN45" s="3" t="n"/>
     </row>
@@ -4964,9 +4956,11 @@
       <c r="AJ46" s="3" t="n"/>
       <c r="AK46" s="3" t="n"/>
       <c r="AL46" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM46" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM46" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN46" s="3" t="n"/>
     </row>
     <row r="47">
@@ -5058,11 +5052,9 @@
       <c r="AJ47" s="3" t="n"/>
       <c r="AK47" s="3" t="n"/>
       <c r="AL47" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM47" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM47" s="10" t="n"/>
       <c r="AN47" s="3" t="n"/>
     </row>
     <row r="48">
@@ -5154,9 +5146,11 @@
       <c r="AJ48" s="3" t="n"/>
       <c r="AK48" s="3" t="n"/>
       <c r="AL48" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM48" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM48" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN48" s="3" t="n"/>
     </row>
     <row r="49">
@@ -5248,9 +5242,11 @@
       <c r="AJ49" s="3" t="n"/>
       <c r="AK49" s="3" t="n"/>
       <c r="AL49" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM49" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM49" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN49" s="3" t="n"/>
     </row>
     <row r="50">
@@ -5342,9 +5338,11 @@
       <c r="AJ50" s="3" t="n"/>
       <c r="AK50" s="3" t="n"/>
       <c r="AL50" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM50" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM50" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN50" s="3" t="n"/>
     </row>
     <row r="51">
@@ -5530,11 +5528,9 @@
       <c r="AJ52" s="3" t="n"/>
       <c r="AK52" s="3" t="n"/>
       <c r="AL52" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM52" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM52" s="10" t="n"/>
       <c r="AN52" s="3" t="n"/>
     </row>
     <row r="53">
@@ -5626,11 +5622,9 @@
       <c r="AJ53" s="3" t="n"/>
       <c r="AK53" s="3" t="n"/>
       <c r="AL53" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM53" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM53" s="10" t="n"/>
       <c r="AN53" s="3" t="n"/>
     </row>
     <row r="54">
@@ -5725,7 +5719,7 @@
         <v>1</v>
       </c>
       <c r="AM54" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN54" s="3" t="n"/>
     </row>
@@ -5818,9 +5812,11 @@
       <c r="AJ55" s="3" t="n"/>
       <c r="AK55" s="3" t="n"/>
       <c r="AL55" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM55" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM55" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN55" s="3" t="n"/>
     </row>
     <row r="56">
@@ -6006,11 +6002,9 @@
       <c r="AJ57" s="3" t="n"/>
       <c r="AK57" s="3" t="n"/>
       <c r="AL57" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM57" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM57" s="10" t="n"/>
       <c r="AN57" s="3" t="n"/>
     </row>
     <row r="58">
@@ -6102,11 +6096,9 @@
       <c r="AJ58" s="3" t="n"/>
       <c r="AK58" s="3" t="n"/>
       <c r="AL58" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM58" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM58" s="10" t="n"/>
       <c r="AN58" s="3" t="n"/>
     </row>
     <row r="59">
@@ -6201,7 +6193,7 @@
         <v>1</v>
       </c>
       <c r="AM59" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN59" s="3" t="n"/>
     </row>
@@ -6294,11 +6286,9 @@
       <c r="AJ60" s="3" t="n"/>
       <c r="AK60" s="3" t="n"/>
       <c r="AL60" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM60" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM60" s="10" t="n"/>
       <c r="AN60" s="3" t="n"/>
     </row>
     <row r="61">
@@ -6484,11 +6474,9 @@
       <c r="AJ62" s="3" t="n"/>
       <c r="AK62" s="3" t="n"/>
       <c r="AL62" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM62" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM62" s="10" t="n"/>
       <c r="AN62" s="3" t="n"/>
     </row>
     <row r="63">
@@ -6580,11 +6568,9 @@
       <c r="AJ63" s="3" t="n"/>
       <c r="AK63" s="3" t="n"/>
       <c r="AL63" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM63" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM63" s="10" t="n"/>
       <c r="AN63" s="3" t="n"/>
     </row>
     <row r="64">
@@ -6679,7 +6665,7 @@
         <v>1</v>
       </c>
       <c r="AM64" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN64" s="3" t="n"/>
     </row>
@@ -6772,11 +6758,9 @@
       <c r="AJ65" s="3" t="n"/>
       <c r="AK65" s="3" t="n"/>
       <c r="AL65" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM65" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM65" s="10" t="n"/>
       <c r="AN65" s="3" t="n"/>
     </row>
     <row r="66">
@@ -6868,11 +6852,9 @@
       <c r="AJ66" s="3" t="n"/>
       <c r="AK66" s="3" t="n"/>
       <c r="AL66" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM66" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM66" s="10" t="n"/>
       <c r="AN66" s="3" t="n"/>
     </row>
     <row r="67">
@@ -6964,9 +6946,11 @@
       <c r="AJ67" s="3" t="n"/>
       <c r="AK67" s="3" t="n"/>
       <c r="AL67" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM67" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM67" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN67" s="3" t="n"/>
     </row>
     <row r="68">
@@ -7058,11 +7042,9 @@
       <c r="AJ68" s="3" t="n"/>
       <c r="AK68" s="3" t="n"/>
       <c r="AL68" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM68" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM68" s="10" t="n"/>
       <c r="AN68" s="3" t="n"/>
     </row>
     <row r="69">
@@ -7154,9 +7136,11 @@
       <c r="AJ69" s="3" t="n"/>
       <c r="AK69" s="3" t="n"/>
       <c r="AL69" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM69" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM69" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN69" s="3" t="n"/>
     </row>
     <row r="70">
@@ -7342,9 +7326,11 @@
       <c r="AJ71" s="3" t="n"/>
       <c r="AK71" s="3" t="n"/>
       <c r="AL71" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM71" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM71" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN71" s="3" t="n"/>
     </row>
     <row r="72">
@@ -7436,9 +7422,11 @@
       <c r="AJ72" s="3" t="n"/>
       <c r="AK72" s="3" t="n"/>
       <c r="AL72" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM72" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM72" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN72" s="3" t="n"/>
     </row>
     <row r="73">
@@ -7624,11 +7612,9 @@
       <c r="AJ74" s="3" t="n"/>
       <c r="AK74" s="3" t="n"/>
       <c r="AL74" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM74" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM74" s="10" t="n"/>
       <c r="AN74" s="3" t="n"/>
     </row>
     <row r="75">
@@ -7720,9 +7706,11 @@
       <c r="AJ75" s="3" t="n"/>
       <c r="AK75" s="3" t="n"/>
       <c r="AL75" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM75" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM75" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN75" s="3" t="n"/>
     </row>
     <row r="76">
@@ -7814,11 +7802,9 @@
       <c r="AJ76" s="3" t="n"/>
       <c r="AK76" s="3" t="n"/>
       <c r="AL76" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM76" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM76" s="10" t="n"/>
       <c r="AN76" s="3" t="n"/>
     </row>
     <row r="77">
@@ -7910,9 +7896,11 @@
       <c r="AJ77" s="3" t="n"/>
       <c r="AK77" s="3" t="n"/>
       <c r="AL77" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM77" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM77" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN77" s="3" t="n"/>
     </row>
     <row r="78">
@@ -8101,7 +8089,7 @@
         <v>1</v>
       </c>
       <c r="AM79" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN79" s="3" t="n"/>
     </row>
@@ -8194,9 +8182,11 @@
       <c r="AJ80" s="3" t="n"/>
       <c r="AK80" s="3" t="n"/>
       <c r="AL80" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM80" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM80" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN80" s="3" t="n"/>
     </row>
     <row r="81">
@@ -8288,11 +8278,9 @@
       <c r="AJ81" s="3" t="n"/>
       <c r="AK81" s="3" t="n"/>
       <c r="AL81" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM81" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM81" s="10" t="n"/>
       <c r="AN81" s="3" t="n"/>
     </row>
     <row r="82">
@@ -8384,9 +8372,11 @@
       <c r="AJ82" s="3" t="n"/>
       <c r="AK82" s="3" t="n"/>
       <c r="AL82" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM82" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM82" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN82" s="3" t="n"/>
     </row>
     <row r="83">
@@ -8478,9 +8468,11 @@
       <c r="AJ83" s="3" t="n"/>
       <c r="AK83" s="3" t="n"/>
       <c r="AL83" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM83" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM83" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN83" s="3" t="n"/>
     </row>
     <row r="84">
@@ -8666,11 +8658,9 @@
       <c r="AJ85" s="3" t="n"/>
       <c r="AK85" s="3" t="n"/>
       <c r="AL85" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM85" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM85" s="10" t="n"/>
       <c r="AN85" s="3" t="n"/>
     </row>
     <row r="86">
@@ -8856,11 +8846,9 @@
       <c r="AJ87" s="3" t="n"/>
       <c r="AK87" s="3" t="n"/>
       <c r="AL87" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM87" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM87" s="10" t="n"/>
       <c r="AN87" s="3" t="n"/>
     </row>
     <row r="88">
@@ -8952,11 +8940,9 @@
       <c r="AJ88" s="3" t="n"/>
       <c r="AK88" s="3" t="n"/>
       <c r="AL88" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM88" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM88" s="10" t="n"/>
       <c r="AN88" s="3" t="n"/>
     </row>
     <row r="89">
@@ -9051,7 +9037,7 @@
         <v>1</v>
       </c>
       <c r="AM89" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN89" s="3" t="n"/>
     </row>
@@ -9241,7 +9227,7 @@
         <v>1</v>
       </c>
       <c r="AM91" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN91" s="3" t="n"/>
     </row>
@@ -9525,7 +9511,7 @@
         <v>1</v>
       </c>
       <c r="AM94" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN94" s="3" t="n"/>
     </row>
@@ -9621,7 +9607,7 @@
         <v>1</v>
       </c>
       <c r="AM95" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN95" s="3" t="n"/>
     </row>
@@ -9714,11 +9700,9 @@
       <c r="AJ96" s="3" t="n"/>
       <c r="AK96" s="3" t="n"/>
       <c r="AL96" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM96" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM96" s="10" t="n"/>
       <c r="AN96" s="3" t="n"/>
     </row>
     <row r="97">
@@ -9810,11 +9794,9 @@
       <c r="AJ97" s="3" t="n"/>
       <c r="AK97" s="3" t="n"/>
       <c r="AL97" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM97" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM97" s="10" t="n"/>
       <c r="AN97" s="3" t="n"/>
     </row>
     <row r="98">
@@ -9906,9 +9888,11 @@
       <c r="AJ98" s="3" t="n"/>
       <c r="AK98" s="3" t="n"/>
       <c r="AL98" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM98" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM98" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN98" s="3" t="n"/>
     </row>
     <row r="99">
@@ -10000,11 +9984,9 @@
       <c r="AJ99" s="3" t="n"/>
       <c r="AK99" s="3" t="n"/>
       <c r="AL99" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM99" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM99" s="10" t="n"/>
       <c r="AN99" s="3" t="n"/>
     </row>
     <row r="100">
@@ -10099,7 +10081,7 @@
         <v>1</v>
       </c>
       <c r="AM100" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN100" s="3" t="n"/>
     </row>
@@ -10286,9 +10268,11 @@
       <c r="AJ102" s="3" t="n"/>
       <c r="AK102" s="3" t="n"/>
       <c r="AL102" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM102" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM102" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN102" s="3" t="n"/>
     </row>
     <row r="103">
@@ -10662,11 +10646,9 @@
       <c r="AJ106" s="3" t="n"/>
       <c r="AK106" s="3" t="n"/>
       <c r="AL106" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM106" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM106" s="10" t="n"/>
       <c r="AN106" s="3" t="n"/>
     </row>
     <row r="107">
@@ -10758,9 +10740,11 @@
       <c r="AJ107" s="3" t="n"/>
       <c r="AK107" s="3" t="n"/>
       <c r="AL107" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM107" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM107" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN107" s="3" t="n"/>
     </row>
     <row r="108">
@@ -10852,9 +10836,11 @@
       <c r="AJ108" s="3" t="n"/>
       <c r="AK108" s="3" t="n"/>
       <c r="AL108" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM108" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM108" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN108" s="3" t="n"/>
     </row>
     <row r="109">
@@ -11040,9 +11026,11 @@
       <c r="AJ110" s="3" t="n"/>
       <c r="AK110" s="3" t="n"/>
       <c r="AL110" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM110" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM110" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN110" s="3" t="n"/>
     </row>
     <row r="111">
@@ -11134,11 +11122,9 @@
       <c r="AJ111" s="3" t="n"/>
       <c r="AK111" s="3" t="n"/>
       <c r="AL111" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM111" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM111" s="10" t="n"/>
       <c r="AN111" s="3" t="n"/>
     </row>
     <row r="112">
@@ -11233,7 +11219,7 @@
         <v>1</v>
       </c>
       <c r="AM112" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN112" s="3" t="n"/>
     </row>
@@ -11326,11 +11312,9 @@
       <c r="AJ113" s="3" t="n"/>
       <c r="AK113" s="3" t="n"/>
       <c r="AL113" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM113" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM113" s="10" t="n"/>
       <c r="AN113" s="3" t="n"/>
     </row>
     <row r="114">
@@ -11425,7 +11409,7 @@
         <v>1</v>
       </c>
       <c r="AM114" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN114" s="3" t="n"/>
     </row>
@@ -11521,7 +11505,7 @@
         <v>1</v>
       </c>
       <c r="AM115" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN115" s="3" t="n"/>
     </row>
@@ -11614,11 +11598,9 @@
       <c r="AJ116" s="3" t="n"/>
       <c r="AK116" s="3" t="n"/>
       <c r="AL116" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM116" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM116" s="10" t="n"/>
       <c r="AN116" s="3" t="n"/>
     </row>
     <row r="117">
@@ -11710,11 +11692,9 @@
       <c r="AJ117" s="3" t="n"/>
       <c r="AK117" s="3" t="n"/>
       <c r="AL117" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM117" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM117" s="10" t="n"/>
       <c r="AN117" s="3" t="n"/>
     </row>
     <row r="118">
@@ -11809,7 +11789,7 @@
         <v>1</v>
       </c>
       <c r="AM118" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN118" s="3" t="n"/>
     </row>
@@ -11902,11 +11882,9 @@
       <c r="AJ119" s="3" t="n"/>
       <c r="AK119" s="3" t="n"/>
       <c r="AL119" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM119" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM119" s="10" t="n"/>
       <c r="AN119" s="3" t="n"/>
     </row>
     <row r="120">
@@ -11998,11 +11976,9 @@
       <c r="AJ120" s="3" t="n"/>
       <c r="AK120" s="3" t="n"/>
       <c r="AL120" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM120" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM120" s="10" t="n"/>
       <c r="AN120" s="3" t="n"/>
     </row>
     <row r="121">
@@ -12097,7 +12073,7 @@
         <v>1</v>
       </c>
       <c r="AM121" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN121" s="3" t="n"/>
     </row>
@@ -12193,7 +12169,7 @@
         <v>1</v>
       </c>
       <c r="AM122" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN122" s="3" t="n"/>
     </row>
@@ -12380,9 +12356,11 @@
       <c r="AJ124" s="3" t="n"/>
       <c r="AK124" s="3" t="n"/>
       <c r="AL124" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM124" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM124" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN124" s="3" t="n"/>
     </row>
     <row r="125">
@@ -12474,9 +12452,11 @@
       <c r="AJ125" s="3" t="n"/>
       <c r="AK125" s="3" t="n"/>
       <c r="AL125" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM125" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM125" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN125" s="3" t="n"/>
     </row>
     <row r="126">
@@ -12568,11 +12548,9 @@
       <c r="AJ126" s="3" t="n"/>
       <c r="AK126" s="3" t="n"/>
       <c r="AL126" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM126" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM126" s="10" t="n"/>
       <c r="AN126" s="3" t="n"/>
     </row>
     <row r="127">
@@ -12664,9 +12642,11 @@
       <c r="AJ127" s="3" t="n"/>
       <c r="AK127" s="3" t="n"/>
       <c r="AL127" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM127" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM127" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN127" s="3" t="n"/>
     </row>
     <row r="128">
@@ -12852,11 +12832,9 @@
       <c r="AJ129" s="3" t="n"/>
       <c r="AK129" s="3" t="n"/>
       <c r="AL129" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM129" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM129" s="10" t="n"/>
       <c r="AN129" s="3" t="n"/>
     </row>
     <row r="130">
@@ -12951,7 +12929,7 @@
         <v>1</v>
       </c>
       <c r="AM130" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN130" s="3" t="n"/>
     </row>
@@ -13047,7 +13025,7 @@
         <v>1</v>
       </c>
       <c r="AM131" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN131" s="3" t="n"/>
     </row>
@@ -13140,11 +13118,9 @@
       <c r="AJ132" s="3" t="n"/>
       <c r="AK132" s="3" t="n"/>
       <c r="AL132" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM132" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM132" s="10" t="n"/>
       <c r="AN132" s="3" t="n"/>
     </row>
     <row r="133">
@@ -13236,9 +13212,11 @@
       <c r="AJ133" s="3" t="n"/>
       <c r="AK133" s="3" t="n"/>
       <c r="AL133" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM133" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM133" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN133" s="3" t="n"/>
     </row>
     <row r="134">
@@ -13330,9 +13308,11 @@
       <c r="AJ134" s="3" t="n"/>
       <c r="AK134" s="3" t="n"/>
       <c r="AL134" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM134" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM134" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN134" s="3" t="n"/>
     </row>
     <row r="135">
@@ -13427,7 +13407,7 @@
         <v>1</v>
       </c>
       <c r="AM135" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN135" s="3" t="n"/>
     </row>
@@ -13520,9 +13500,11 @@
       <c r="AJ136" s="3" t="n"/>
       <c r="AK136" s="3" t="n"/>
       <c r="AL136" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM136" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM136" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN136" s="3" t="n"/>
     </row>
     <row r="137">
@@ -13614,11 +13596,9 @@
       <c r="AJ137" s="3" t="n"/>
       <c r="AK137" s="3" t="n"/>
       <c r="AL137" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM137" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM137" s="10" t="n"/>
       <c r="AN137" s="3" t="n"/>
     </row>
     <row r="138">
@@ -13713,7 +13693,7 @@
         <v>1</v>
       </c>
       <c r="AM138" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN138" s="3" t="n"/>
     </row>
@@ -13809,7 +13789,7 @@
         <v>1</v>
       </c>
       <c r="AM139" s="10" t="n">
-        <v>46216.62358983864</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN139" s="3" t="n"/>
     </row>
@@ -13905,7 +13885,7 @@
         <v>1</v>
       </c>
       <c r="AM140" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN140" s="3" t="n"/>
     </row>
@@ -13998,11 +13978,9 @@
       <c r="AJ141" s="3" t="n"/>
       <c r="AK141" s="3" t="n"/>
       <c r="AL141" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM141" s="10" t="n">
-        <v>46216.62358983864</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM141" s="10" t="n"/>
       <c r="AN141" s="3" t="n"/>
     </row>
     <row r="142">
@@ -14094,9 +14072,11 @@
       <c r="AJ142" s="3" t="n"/>
       <c r="AK142" s="3" t="n"/>
       <c r="AL142" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM142" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM142" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN142" s="3" t="n"/>
     </row>
     <row r="143">
@@ -14188,11 +14168,9 @@
       <c r="AJ143" s="3" t="n"/>
       <c r="AK143" s="3" t="n"/>
       <c r="AL143" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM143" s="10" t="n">
-        <v>46216.62358892361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM143" s="10" t="n"/>
       <c r="AN143" s="3" t="n"/>
     </row>
     <row r="144">
@@ -14284,9 +14262,11 @@
       <c r="AJ144" s="3" t="n"/>
       <c r="AK144" s="3" t="n"/>
       <c r="AL144" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM144" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM144" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN144" s="3" t="n"/>
     </row>
     <row r="145">
@@ -14378,9 +14358,11 @@
       <c r="AJ145" s="3" t="n"/>
       <c r="AK145" s="3" t="n"/>
       <c r="AL145" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM145" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM145" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN145" s="3" t="n"/>
     </row>
     <row r="146">
@@ -14472,9 +14454,11 @@
       <c r="AJ146" s="3" t="n"/>
       <c r="AK146" s="3" t="n"/>
       <c r="AL146" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM146" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM146" s="10" t="n">
+        <v>46217.35774947917</v>
+      </c>
       <c r="AN146" s="3" t="n"/>
     </row>
     <row r="147">
@@ -14566,9 +14550,11 @@
       <c r="AJ147" s="3" t="n"/>
       <c r="AK147" s="3" t="n"/>
       <c r="AL147" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM147" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM147" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN147" s="3" t="n"/>
     </row>
     <row r="148">
@@ -14663,7 +14649,7 @@
         <v>1</v>
       </c>
       <c r="AM148" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35774947917</v>
       </c>
       <c r="AN148" s="3" t="n"/>
     </row>
@@ -14759,7 +14745,7 @@
         <v>1</v>
       </c>
       <c r="AM149" s="10" t="n">
-        <v>46216.62358892361</v>
+        <v>46217.35775057751</v>
       </c>
       <c r="AN149" s="3" t="n"/>
     </row>
@@ -14852,9 +14838,11 @@
       <c r="AJ150" s="3" t="n"/>
       <c r="AK150" s="3" t="n"/>
       <c r="AL150" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM150" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM150" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN150" s="3" t="n"/>
     </row>
     <row r="151">
@@ -14946,9 +14934,11 @@
       <c r="AJ151" s="3" t="n"/>
       <c r="AK151" s="3" t="n"/>
       <c r="AL151" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM151" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM151" s="10" t="n">
+        <v>46217.35775057751</v>
+      </c>
       <c r="AN151" s="3" t="n"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
utilities testing suite + remaining notes
</commit_message>
<xml_diff>
--- a/helpers/testing/test_output.xlsx
+++ b/helpers/testing/test_output.xlsx
@@ -967,7 +967,7 @@
         <v>1</v>
       </c>
       <c r="AM4" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN4" s="3" t="n"/>
     </row>
@@ -1060,11 +1060,9 @@
       <c r="AJ5" s="3" t="n"/>
       <c r="AK5" s="3" t="n"/>
       <c r="AL5" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM5" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM5" s="10" t="n"/>
       <c r="AN5" s="3" t="n"/>
     </row>
     <row r="6">
@@ -1156,9 +1154,11 @@
       <c r="AJ6" s="3" t="n"/>
       <c r="AK6" s="3" t="n"/>
       <c r="AL6" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM6" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM6" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN6" s="3" t="n"/>
     </row>
     <row r="7">
@@ -1344,9 +1344,11 @@
       <c r="AJ8" s="3" t="n"/>
       <c r="AK8" s="3" t="n"/>
       <c r="AL8" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM8" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM8" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN8" s="3" t="n"/>
     </row>
     <row r="9">
@@ -1532,9 +1534,11 @@
       <c r="AJ10" s="3" t="n"/>
       <c r="AK10" s="3" t="n"/>
       <c r="AL10" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM10" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM10" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN10" s="3" t="n"/>
     </row>
     <row r="11">
@@ -1626,11 +1630,9 @@
       <c r="AJ11" s="3" t="n"/>
       <c r="AK11" s="3" t="n"/>
       <c r="AL11" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM11" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM11" s="10" t="n"/>
       <c r="AN11" s="3" t="n"/>
     </row>
     <row r="12">
@@ -1725,7 +1727,7 @@
         <v>1</v>
       </c>
       <c r="AM12" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN12" s="3" t="n"/>
     </row>
@@ -1821,7 +1823,7 @@
         <v>1</v>
       </c>
       <c r="AM13" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN13" s="3" t="n"/>
     </row>
@@ -1917,7 +1919,7 @@
         <v>1</v>
       </c>
       <c r="AM14" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN14" s="3" t="n"/>
     </row>
@@ -2010,9 +2012,11 @@
       <c r="AJ15" s="3" t="n"/>
       <c r="AK15" s="3" t="n"/>
       <c r="AL15" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM15" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM15" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN15" s="3" t="n"/>
     </row>
     <row r="16">
@@ -2107,7 +2111,7 @@
         <v>1</v>
       </c>
       <c r="AM16" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN16" s="3" t="n"/>
     </row>
@@ -2200,9 +2204,11 @@
       <c r="AJ17" s="3" t="n"/>
       <c r="AK17" s="3" t="n"/>
       <c r="AL17" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM17" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM17" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN17" s="3" t="n"/>
     </row>
     <row r="18">
@@ -2294,11 +2300,9 @@
       <c r="AJ18" s="3" t="n"/>
       <c r="AK18" s="3" t="n"/>
       <c r="AL18" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM18" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM18" s="10" t="n"/>
       <c r="AN18" s="3" t="n"/>
     </row>
     <row r="19">
@@ -2390,11 +2394,9 @@
       <c r="AJ19" s="3" t="n"/>
       <c r="AK19" s="3" t="n"/>
       <c r="AL19" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM19" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM19" s="10" t="n"/>
       <c r="AN19" s="3" t="n"/>
     </row>
     <row r="20">
@@ -2486,9 +2488,11 @@
       <c r="AJ20" s="3" t="n"/>
       <c r="AK20" s="3" t="n"/>
       <c r="AL20" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM20" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM20" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN20" s="3" t="n"/>
     </row>
     <row r="21">
@@ -2580,9 +2584,11 @@
       <c r="AJ21" s="3" t="n"/>
       <c r="AK21" s="3" t="n"/>
       <c r="AL21" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM21" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM21" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN21" s="3" t="n"/>
     </row>
     <row r="22">
@@ -2674,11 +2680,9 @@
       <c r="AJ22" s="3" t="n"/>
       <c r="AK22" s="3" t="n"/>
       <c r="AL22" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM22" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM22" s="10" t="n"/>
       <c r="AN22" s="3" t="n"/>
     </row>
     <row r="23">
@@ -2864,11 +2868,9 @@
       <c r="AJ24" s="3" t="n"/>
       <c r="AK24" s="3" t="n"/>
       <c r="AL24" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM24" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM24" s="10" t="n"/>
       <c r="AN24" s="3" t="n"/>
     </row>
     <row r="25">
@@ -2963,7 +2965,7 @@
         <v>1</v>
       </c>
       <c r="AM25" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN25" s="3" t="n"/>
     </row>
@@ -3341,7 +3343,7 @@
         <v>1</v>
       </c>
       <c r="AM29" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN29" s="3" t="n"/>
     </row>
@@ -3531,7 +3533,7 @@
         <v>1</v>
       </c>
       <c r="AM31" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN31" s="3" t="n"/>
     </row>
@@ -3627,7 +3629,7 @@
         <v>1</v>
       </c>
       <c r="AM32" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN32" s="3" t="n"/>
     </row>
@@ -3723,7 +3725,7 @@
         <v>1</v>
       </c>
       <c r="AM33" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN33" s="3" t="n"/>
     </row>
@@ -3913,7 +3915,7 @@
         <v>1</v>
       </c>
       <c r="AM35" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN35" s="3" t="n"/>
     </row>
@@ -4100,11 +4102,9 @@
       <c r="AJ37" s="3" t="n"/>
       <c r="AK37" s="3" t="n"/>
       <c r="AL37" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM37" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM37" s="10" t="n"/>
       <c r="AN37" s="3" t="n"/>
     </row>
     <row r="38">
@@ -4196,9 +4196,11 @@
       <c r="AJ38" s="3" t="n"/>
       <c r="AK38" s="3" t="n"/>
       <c r="AL38" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM38" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM38" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN38" s="3" t="n"/>
     </row>
     <row r="39">
@@ -4290,9 +4292,11 @@
       <c r="AJ39" s="3" t="n"/>
       <c r="AK39" s="3" t="n"/>
       <c r="AL39" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM39" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM39" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN39" s="3" t="n"/>
     </row>
     <row r="40">
@@ -4387,7 +4391,7 @@
         <v>1</v>
       </c>
       <c r="AM40" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN40" s="3" t="n"/>
     </row>
@@ -4480,11 +4484,9 @@
       <c r="AJ41" s="3" t="n"/>
       <c r="AK41" s="3" t="n"/>
       <c r="AL41" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM41" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM41" s="10" t="n"/>
       <c r="AN41" s="3" t="n"/>
     </row>
     <row r="42">
@@ -4579,7 +4581,7 @@
         <v>1</v>
       </c>
       <c r="AM42" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN42" s="3" t="n"/>
     </row>
@@ -4860,11 +4862,9 @@
       <c r="AJ45" s="3" t="n"/>
       <c r="AK45" s="3" t="n"/>
       <c r="AL45" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM45" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM45" s="10" t="n"/>
       <c r="AN45" s="3" t="n"/>
     </row>
     <row r="46">
@@ -4956,11 +4956,9 @@
       <c r="AJ46" s="3" t="n"/>
       <c r="AK46" s="3" t="n"/>
       <c r="AL46" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM46" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM46" s="10" t="n"/>
       <c r="AN46" s="3" t="n"/>
     </row>
     <row r="47">
@@ -5052,9 +5050,11 @@
       <c r="AJ47" s="3" t="n"/>
       <c r="AK47" s="3" t="n"/>
       <c r="AL47" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM47" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM47" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN47" s="3" t="n"/>
     </row>
     <row r="48">
@@ -5149,7 +5149,7 @@
         <v>1</v>
       </c>
       <c r="AM48" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN48" s="3" t="n"/>
     </row>
@@ -5242,11 +5242,9 @@
       <c r="AJ49" s="3" t="n"/>
       <c r="AK49" s="3" t="n"/>
       <c r="AL49" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM49" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM49" s="10" t="n"/>
       <c r="AN49" s="3" t="n"/>
     </row>
     <row r="50">
@@ -5341,7 +5339,7 @@
         <v>1</v>
       </c>
       <c r="AM50" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN50" s="3" t="n"/>
     </row>
@@ -5528,9 +5526,11 @@
       <c r="AJ52" s="3" t="n"/>
       <c r="AK52" s="3" t="n"/>
       <c r="AL52" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM52" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM52" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN52" s="3" t="n"/>
     </row>
     <row r="53">
@@ -5719,7 +5719,7 @@
         <v>1</v>
       </c>
       <c r="AM54" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN54" s="3" t="n"/>
     </row>
@@ -5812,11 +5812,9 @@
       <c r="AJ55" s="3" t="n"/>
       <c r="AK55" s="3" t="n"/>
       <c r="AL55" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM55" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM55" s="10" t="n"/>
       <c r="AN55" s="3" t="n"/>
     </row>
     <row r="56">
@@ -5908,9 +5906,11 @@
       <c r="AJ56" s="3" t="n"/>
       <c r="AK56" s="3" t="n"/>
       <c r="AL56" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM56" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM56" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN56" s="3" t="n"/>
     </row>
     <row r="57">
@@ -6190,11 +6190,9 @@
       <c r="AJ59" s="3" t="n"/>
       <c r="AK59" s="3" t="n"/>
       <c r="AL59" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM59" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM59" s="10" t="n"/>
       <c r="AN59" s="3" t="n"/>
     </row>
     <row r="60">
@@ -6286,9 +6284,11 @@
       <c r="AJ60" s="3" t="n"/>
       <c r="AK60" s="3" t="n"/>
       <c r="AL60" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM60" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM60" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN60" s="3" t="n"/>
     </row>
     <row r="61">
@@ -6568,9 +6568,11 @@
       <c r="AJ63" s="3" t="n"/>
       <c r="AK63" s="3" t="n"/>
       <c r="AL63" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM63" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM63" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN63" s="3" t="n"/>
     </row>
     <row r="64">
@@ -6665,7 +6667,7 @@
         <v>1</v>
       </c>
       <c r="AM64" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN64" s="3" t="n"/>
     </row>
@@ -6758,9 +6760,11 @@
       <c r="AJ65" s="3" t="n"/>
       <c r="AK65" s="3" t="n"/>
       <c r="AL65" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM65" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM65" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN65" s="3" t="n"/>
     </row>
     <row r="66">
@@ -6852,9 +6856,11 @@
       <c r="AJ66" s="3" t="n"/>
       <c r="AK66" s="3" t="n"/>
       <c r="AL66" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM66" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM66" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN66" s="3" t="n"/>
     </row>
     <row r="67">
@@ -6946,11 +6952,9 @@
       <c r="AJ67" s="3" t="n"/>
       <c r="AK67" s="3" t="n"/>
       <c r="AL67" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM67" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM67" s="10" t="n"/>
       <c r="AN67" s="3" t="n"/>
     </row>
     <row r="68">
@@ -7139,7 +7143,7 @@
         <v>1</v>
       </c>
       <c r="AM69" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN69" s="3" t="n"/>
     </row>
@@ -7232,9 +7236,11 @@
       <c r="AJ70" s="3" t="n"/>
       <c r="AK70" s="3" t="n"/>
       <c r="AL70" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM70" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM70" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN70" s="3" t="n"/>
     </row>
     <row r="71">
@@ -7326,11 +7332,9 @@
       <c r="AJ71" s="3" t="n"/>
       <c r="AK71" s="3" t="n"/>
       <c r="AL71" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM71" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM71" s="10" t="n"/>
       <c r="AN71" s="3" t="n"/>
     </row>
     <row r="72">
@@ -7422,11 +7426,9 @@
       <c r="AJ72" s="3" t="n"/>
       <c r="AK72" s="3" t="n"/>
       <c r="AL72" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM72" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM72" s="10" t="n"/>
       <c r="AN72" s="3" t="n"/>
     </row>
     <row r="73">
@@ -7518,9 +7520,11 @@
       <c r="AJ73" s="3" t="n"/>
       <c r="AK73" s="3" t="n"/>
       <c r="AL73" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM73" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM73" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN73" s="3" t="n"/>
     </row>
     <row r="74">
@@ -7612,9 +7616,11 @@
       <c r="AJ74" s="3" t="n"/>
       <c r="AK74" s="3" t="n"/>
       <c r="AL74" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM74" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM74" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN74" s="3" t="n"/>
     </row>
     <row r="75">
@@ -7706,11 +7712,9 @@
       <c r="AJ75" s="3" t="n"/>
       <c r="AK75" s="3" t="n"/>
       <c r="AL75" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM75" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM75" s="10" t="n"/>
       <c r="AN75" s="3" t="n"/>
     </row>
     <row r="76">
@@ -7896,11 +7900,9 @@
       <c r="AJ77" s="3" t="n"/>
       <c r="AK77" s="3" t="n"/>
       <c r="AL77" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM77" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM77" s="10" t="n"/>
       <c r="AN77" s="3" t="n"/>
     </row>
     <row r="78">
@@ -8086,11 +8088,9 @@
       <c r="AJ79" s="3" t="n"/>
       <c r="AK79" s="3" t="n"/>
       <c r="AL79" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM79" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM79" s="10" t="n"/>
       <c r="AN79" s="3" t="n"/>
     </row>
     <row r="80">
@@ -8185,7 +8185,7 @@
         <v>1</v>
       </c>
       <c r="AM80" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN80" s="3" t="n"/>
     </row>
@@ -8372,11 +8372,9 @@
       <c r="AJ82" s="3" t="n"/>
       <c r="AK82" s="3" t="n"/>
       <c r="AL82" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM82" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM82" s="10" t="n"/>
       <c r="AN82" s="3" t="n"/>
     </row>
     <row r="83">
@@ -8471,7 +8469,7 @@
         <v>1</v>
       </c>
       <c r="AM83" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN83" s="3" t="n"/>
     </row>
@@ -8940,9 +8938,11 @@
       <c r="AJ88" s="3" t="n"/>
       <c r="AK88" s="3" t="n"/>
       <c r="AL88" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM88" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM88" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN88" s="3" t="n"/>
     </row>
     <row r="89">
@@ -9037,7 +9037,7 @@
         <v>1</v>
       </c>
       <c r="AM89" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN89" s="3" t="n"/>
     </row>
@@ -9130,9 +9130,11 @@
       <c r="AJ90" s="3" t="n"/>
       <c r="AK90" s="3" t="n"/>
       <c r="AL90" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM90" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM90" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN90" s="3" t="n"/>
     </row>
     <row r="91">
@@ -9227,7 +9229,7 @@
         <v>1</v>
       </c>
       <c r="AM91" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN91" s="3" t="n"/>
     </row>
@@ -9511,7 +9513,7 @@
         <v>1</v>
       </c>
       <c r="AM94" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN94" s="3" t="n"/>
     </row>
@@ -9604,11 +9606,9 @@
       <c r="AJ95" s="3" t="n"/>
       <c r="AK95" s="3" t="n"/>
       <c r="AL95" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM95" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM95" s="10" t="n"/>
       <c r="AN95" s="3" t="n"/>
     </row>
     <row r="96">
@@ -9888,11 +9888,9 @@
       <c r="AJ98" s="3" t="n"/>
       <c r="AK98" s="3" t="n"/>
       <c r="AL98" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM98" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM98" s="10" t="n"/>
       <c r="AN98" s="3" t="n"/>
     </row>
     <row r="99">
@@ -10081,7 +10079,7 @@
         <v>1</v>
       </c>
       <c r="AM100" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN100" s="3" t="n"/>
     </row>
@@ -10271,7 +10269,7 @@
         <v>1</v>
       </c>
       <c r="AM102" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN102" s="3" t="n"/>
     </row>
@@ -10740,11 +10738,9 @@
       <c r="AJ107" s="3" t="n"/>
       <c r="AK107" s="3" t="n"/>
       <c r="AL107" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM107" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM107" s="10" t="n"/>
       <c r="AN107" s="3" t="n"/>
     </row>
     <row r="108">
@@ -10836,11 +10832,9 @@
       <c r="AJ108" s="3" t="n"/>
       <c r="AK108" s="3" t="n"/>
       <c r="AL108" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM108" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM108" s="10" t="n"/>
       <c r="AN108" s="3" t="n"/>
     </row>
     <row r="109">
@@ -10932,9 +10926,11 @@
       <c r="AJ109" s="3" t="n"/>
       <c r="AK109" s="3" t="n"/>
       <c r="AL109" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM109" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM109" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN109" s="3" t="n"/>
     </row>
     <row r="110">
@@ -11026,11 +11022,9 @@
       <c r="AJ110" s="3" t="n"/>
       <c r="AK110" s="3" t="n"/>
       <c r="AL110" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM110" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM110" s="10" t="n"/>
       <c r="AN110" s="3" t="n"/>
     </row>
     <row r="111">
@@ -11216,11 +11210,9 @@
       <c r="AJ112" s="3" t="n"/>
       <c r="AK112" s="3" t="n"/>
       <c r="AL112" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM112" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM112" s="10" t="n"/>
       <c r="AN112" s="3" t="n"/>
     </row>
     <row r="113">
@@ -11312,9 +11304,11 @@
       <c r="AJ113" s="3" t="n"/>
       <c r="AK113" s="3" t="n"/>
       <c r="AL113" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM113" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM113" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN113" s="3" t="n"/>
     </row>
     <row r="114">
@@ -11406,11 +11400,9 @@
       <c r="AJ114" s="3" t="n"/>
       <c r="AK114" s="3" t="n"/>
       <c r="AL114" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM114" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM114" s="10" t="n"/>
       <c r="AN114" s="3" t="n"/>
     </row>
     <row r="115">
@@ -11505,7 +11497,7 @@
         <v>1</v>
       </c>
       <c r="AM115" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN115" s="3" t="n"/>
     </row>
@@ -11786,11 +11778,9 @@
       <c r="AJ118" s="3" t="n"/>
       <c r="AK118" s="3" t="n"/>
       <c r="AL118" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM118" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM118" s="10" t="n"/>
       <c r="AN118" s="3" t="n"/>
     </row>
     <row r="119">
@@ -11882,9 +11872,11 @@
       <c r="AJ119" s="3" t="n"/>
       <c r="AK119" s="3" t="n"/>
       <c r="AL119" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM119" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM119" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN119" s="3" t="n"/>
     </row>
     <row r="120">
@@ -12073,7 +12065,7 @@
         <v>1</v>
       </c>
       <c r="AM121" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN121" s="3" t="n"/>
     </row>
@@ -12169,7 +12161,7 @@
         <v>1</v>
       </c>
       <c r="AM122" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN122" s="3" t="n"/>
     </row>
@@ -12262,9 +12254,11 @@
       <c r="AJ123" s="3" t="n"/>
       <c r="AK123" s="3" t="n"/>
       <c r="AL123" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM123" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM123" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN123" s="3" t="n"/>
     </row>
     <row r="124">
@@ -12359,7 +12353,7 @@
         <v>1</v>
       </c>
       <c r="AM124" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN124" s="3" t="n"/>
     </row>
@@ -12452,11 +12446,9 @@
       <c r="AJ125" s="3" t="n"/>
       <c r="AK125" s="3" t="n"/>
       <c r="AL125" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM125" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM125" s="10" t="n"/>
       <c r="AN125" s="3" t="n"/>
     </row>
     <row r="126">
@@ -12548,9 +12540,11 @@
       <c r="AJ126" s="3" t="n"/>
       <c r="AK126" s="3" t="n"/>
       <c r="AL126" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM126" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM126" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN126" s="3" t="n"/>
     </row>
     <row r="127">
@@ -12642,11 +12636,9 @@
       <c r="AJ127" s="3" t="n"/>
       <c r="AK127" s="3" t="n"/>
       <c r="AL127" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM127" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM127" s="10" t="n"/>
       <c r="AN127" s="3" t="n"/>
     </row>
     <row r="128">
@@ -12929,7 +12921,7 @@
         <v>1</v>
       </c>
       <c r="AM130" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN130" s="3" t="n"/>
     </row>
@@ -13022,11 +13014,9 @@
       <c r="AJ131" s="3" t="n"/>
       <c r="AK131" s="3" t="n"/>
       <c r="AL131" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM131" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM131" s="10" t="n"/>
       <c r="AN131" s="3" t="n"/>
     </row>
     <row r="132">
@@ -13118,9 +13108,11 @@
       <c r="AJ132" s="3" t="n"/>
       <c r="AK132" s="3" t="n"/>
       <c r="AL132" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM132" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM132" s="10" t="n">
+        <v>46217.4577819237</v>
+      </c>
       <c r="AN132" s="3" t="n"/>
     </row>
     <row r="133">
@@ -13215,7 +13207,7 @@
         <v>1</v>
       </c>
       <c r="AM133" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.4577819237</v>
       </c>
       <c r="AN133" s="3" t="n"/>
     </row>
@@ -13308,11 +13300,9 @@
       <c r="AJ134" s="3" t="n"/>
       <c r="AK134" s="3" t="n"/>
       <c r="AL134" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM134" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM134" s="10" t="n"/>
       <c r="AN134" s="3" t="n"/>
     </row>
     <row r="135">
@@ -13404,11 +13394,9 @@
       <c r="AJ135" s="3" t="n"/>
       <c r="AK135" s="3" t="n"/>
       <c r="AL135" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM135" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM135" s="10" t="n"/>
       <c r="AN135" s="3" t="n"/>
     </row>
     <row r="136">
@@ -13500,11 +13488,9 @@
       <c r="AJ136" s="3" t="n"/>
       <c r="AK136" s="3" t="n"/>
       <c r="AL136" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM136" s="10" t="n">
-        <v>46217.35774947917</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM136" s="10" t="n"/>
       <c r="AN136" s="3" t="n"/>
     </row>
     <row r="137">
@@ -13596,9 +13582,11 @@
       <c r="AJ137" s="3" t="n"/>
       <c r="AK137" s="3" t="n"/>
       <c r="AL137" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM137" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM137" s="10" t="n">
+        <v>46217.45778064815</v>
+      </c>
       <c r="AN137" s="3" t="n"/>
     </row>
     <row r="138">
@@ -13693,7 +13681,7 @@
         <v>1</v>
       </c>
       <c r="AM138" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN138" s="3" t="n"/>
     </row>
@@ -13789,7 +13777,7 @@
         <v>1</v>
       </c>
       <c r="AM139" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN139" s="3" t="n"/>
     </row>
@@ -13882,11 +13870,9 @@
       <c r="AJ140" s="3" t="n"/>
       <c r="AK140" s="3" t="n"/>
       <c r="AL140" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM140" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM140" s="10" t="n"/>
       <c r="AN140" s="3" t="n"/>
     </row>
     <row r="141">
@@ -14075,7 +14061,7 @@
         <v>1</v>
       </c>
       <c r="AM142" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778210896</v>
       </c>
       <c r="AN142" s="3" t="n"/>
     </row>
@@ -14262,11 +14248,9 @@
       <c r="AJ144" s="3" t="n"/>
       <c r="AK144" s="3" t="n"/>
       <c r="AL144" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM144" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM144" s="10" t="n"/>
       <c r="AN144" s="3" t="n"/>
     </row>
     <row r="145">
@@ -14361,7 +14345,7 @@
         <v>1</v>
       </c>
       <c r="AM145" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778210896</v>
       </c>
       <c r="AN145" s="3" t="n"/>
     </row>
@@ -14457,7 +14441,7 @@
         <v>1</v>
       </c>
       <c r="AM146" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778210896</v>
       </c>
       <c r="AN146" s="3" t="n"/>
     </row>
@@ -14553,7 +14537,7 @@
         <v>1</v>
       </c>
       <c r="AM147" s="10" t="n">
-        <v>46217.35775057751</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN147" s="3" t="n"/>
     </row>
@@ -14649,7 +14633,7 @@
         <v>1</v>
       </c>
       <c r="AM148" s="10" t="n">
-        <v>46217.35774947917</v>
+        <v>46217.45778064815</v>
       </c>
       <c r="AN148" s="3" t="n"/>
     </row>
@@ -14742,11 +14726,9 @@
       <c r="AJ149" s="3" t="n"/>
       <c r="AK149" s="3" t="n"/>
       <c r="AL149" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM149" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM149" s="10" t="n"/>
       <c r="AN149" s="3" t="n"/>
     </row>
     <row r="150">
@@ -14838,11 +14820,9 @@
       <c r="AJ150" s="3" t="n"/>
       <c r="AK150" s="3" t="n"/>
       <c r="AL150" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM150" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM150" s="10" t="n"/>
       <c r="AN150" s="3" t="n"/>
     </row>
     <row r="151">
@@ -14934,11 +14914,9 @@
       <c r="AJ151" s="3" t="n"/>
       <c r="AK151" s="3" t="n"/>
       <c r="AL151" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM151" s="10" t="n">
-        <v>46217.35775057751</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM151" s="10" t="n"/>
       <c r="AN151" s="3" t="n"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
wrapping up major test cases + comments
</commit_message>
<xml_diff>
--- a/helpers/testing/test_output.xlsx
+++ b/helpers/testing/test_output.xlsx
@@ -776,9 +776,11 @@
       <c r="AJ2" s="3" t="n"/>
       <c r="AK2" s="3" t="n"/>
       <c r="AL2" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM2" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM2" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN2" s="3" t="n"/>
     </row>
     <row r="3">
@@ -964,11 +966,9 @@
       <c r="AJ4" s="3" t="n"/>
       <c r="AK4" s="3" t="n"/>
       <c r="AL4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM4" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM4" s="10" t="n"/>
       <c r="AN4" s="3" t="n"/>
     </row>
     <row r="5">
@@ -1154,11 +1154,9 @@
       <c r="AJ6" s="3" t="n"/>
       <c r="AK6" s="3" t="n"/>
       <c r="AL6" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM6" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM6" s="10" t="n"/>
       <c r="AN6" s="3" t="n"/>
     </row>
     <row r="7">
@@ -1250,9 +1248,11 @@
       <c r="AJ7" s="3" t="n"/>
       <c r="AK7" s="3" t="n"/>
       <c r="AL7" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM7" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM7" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN7" s="3" t="n"/>
     </row>
     <row r="8">
@@ -1344,11 +1344,9 @@
       <c r="AJ8" s="3" t="n"/>
       <c r="AK8" s="3" t="n"/>
       <c r="AL8" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM8" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM8" s="10" t="n"/>
       <c r="AN8" s="3" t="n"/>
     </row>
     <row r="9">
@@ -1534,11 +1532,9 @@
       <c r="AJ10" s="3" t="n"/>
       <c r="AK10" s="3" t="n"/>
       <c r="AL10" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM10" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM10" s="10" t="n"/>
       <c r="AN10" s="3" t="n"/>
     </row>
     <row r="11">
@@ -1727,7 +1723,7 @@
         <v>1</v>
       </c>
       <c r="AM12" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN12" s="3" t="n"/>
     </row>
@@ -1820,11 +1816,9 @@
       <c r="AJ13" s="3" t="n"/>
       <c r="AK13" s="3" t="n"/>
       <c r="AL13" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM13" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM13" s="10" t="n"/>
       <c r="AN13" s="3" t="n"/>
     </row>
     <row r="14">
@@ -1919,7 +1913,7 @@
         <v>1</v>
       </c>
       <c r="AM14" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN14" s="3" t="n"/>
     </row>
@@ -2015,7 +2009,7 @@
         <v>1</v>
       </c>
       <c r="AM15" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN15" s="3" t="n"/>
     </row>
@@ -2111,7 +2105,7 @@
         <v>1</v>
       </c>
       <c r="AM16" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN16" s="3" t="n"/>
     </row>
@@ -2207,7 +2201,7 @@
         <v>1</v>
       </c>
       <c r="AM17" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN17" s="3" t="n"/>
     </row>
@@ -2394,9 +2388,11 @@
       <c r="AJ19" s="3" t="n"/>
       <c r="AK19" s="3" t="n"/>
       <c r="AL19" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM19" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM19" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN19" s="3" t="n"/>
     </row>
     <row r="20">
@@ -2488,11 +2484,9 @@
       <c r="AJ20" s="3" t="n"/>
       <c r="AK20" s="3" t="n"/>
       <c r="AL20" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM20" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM20" s="10" t="n"/>
       <c r="AN20" s="3" t="n"/>
     </row>
     <row r="21">
@@ -2584,11 +2578,9 @@
       <c r="AJ21" s="3" t="n"/>
       <c r="AK21" s="3" t="n"/>
       <c r="AL21" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM21" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM21" s="10" t="n"/>
       <c r="AN21" s="3" t="n"/>
     </row>
     <row r="22">
@@ -2868,9 +2860,11 @@
       <c r="AJ24" s="3" t="n"/>
       <c r="AK24" s="3" t="n"/>
       <c r="AL24" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM24" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM24" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN24" s="3" t="n"/>
     </row>
     <row r="25">
@@ -2962,11 +2956,9 @@
       <c r="AJ25" s="3" t="n"/>
       <c r="AK25" s="3" t="n"/>
       <c r="AL25" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM25" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM25" s="10" t="n"/>
       <c r="AN25" s="3" t="n"/>
     </row>
     <row r="26">
@@ -3340,11 +3332,9 @@
       <c r="AJ29" s="3" t="n"/>
       <c r="AK29" s="3" t="n"/>
       <c r="AL29" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM29" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM29" s="10" t="n"/>
       <c r="AN29" s="3" t="n"/>
     </row>
     <row r="30">
@@ -3530,11 +3520,9 @@
       <c r="AJ31" s="3" t="n"/>
       <c r="AK31" s="3" t="n"/>
       <c r="AL31" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM31" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM31" s="10" t="n"/>
       <c r="AN31" s="3" t="n"/>
     </row>
     <row r="32">
@@ -3626,11 +3614,9 @@
       <c r="AJ32" s="3" t="n"/>
       <c r="AK32" s="3" t="n"/>
       <c r="AL32" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM32" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM32" s="10" t="n"/>
       <c r="AN32" s="3" t="n"/>
     </row>
     <row r="33">
@@ -3722,11 +3708,9 @@
       <c r="AJ33" s="3" t="n"/>
       <c r="AK33" s="3" t="n"/>
       <c r="AL33" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM33" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM33" s="10" t="n"/>
       <c r="AN33" s="3" t="n"/>
     </row>
     <row r="34">
@@ -3915,7 +3899,7 @@
         <v>1</v>
       </c>
       <c r="AM35" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN35" s="3" t="n"/>
     </row>
@@ -4008,9 +3992,11 @@
       <c r="AJ36" s="3" t="n"/>
       <c r="AK36" s="3" t="n"/>
       <c r="AL36" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM36" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM36" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN36" s="3" t="n"/>
     </row>
     <row r="37">
@@ -4199,7 +4185,7 @@
         <v>1</v>
       </c>
       <c r="AM38" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN38" s="3" t="n"/>
     </row>
@@ -4295,7 +4281,7 @@
         <v>1</v>
       </c>
       <c r="AM39" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN39" s="3" t="n"/>
     </row>
@@ -4388,11 +4374,9 @@
       <c r="AJ40" s="3" t="n"/>
       <c r="AK40" s="3" t="n"/>
       <c r="AL40" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM40" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM40" s="10" t="n"/>
       <c r="AN40" s="3" t="n"/>
     </row>
     <row r="41">
@@ -4484,9 +4468,11 @@
       <c r="AJ41" s="3" t="n"/>
       <c r="AK41" s="3" t="n"/>
       <c r="AL41" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM41" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM41" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN41" s="3" t="n"/>
     </row>
     <row r="42">
@@ -4581,7 +4567,7 @@
         <v>1</v>
       </c>
       <c r="AM42" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN42" s="3" t="n"/>
     </row>
@@ -4674,9 +4660,11 @@
       <c r="AJ43" s="3" t="n"/>
       <c r="AK43" s="3" t="n"/>
       <c r="AL43" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM43" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM43" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN43" s="3" t="n"/>
     </row>
     <row r="44">
@@ -4768,9 +4756,11 @@
       <c r="AJ44" s="3" t="n"/>
       <c r="AK44" s="3" t="n"/>
       <c r="AL44" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM44" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM44" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN44" s="3" t="n"/>
     </row>
     <row r="45">
@@ -4862,9 +4852,11 @@
       <c r="AJ45" s="3" t="n"/>
       <c r="AK45" s="3" t="n"/>
       <c r="AL45" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM45" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM45" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN45" s="3" t="n"/>
     </row>
     <row r="46">
@@ -5050,11 +5042,9 @@
       <c r="AJ47" s="3" t="n"/>
       <c r="AK47" s="3" t="n"/>
       <c r="AL47" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM47" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM47" s="10" t="n"/>
       <c r="AN47" s="3" t="n"/>
     </row>
     <row r="48">
@@ -5149,7 +5139,7 @@
         <v>1</v>
       </c>
       <c r="AM48" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN48" s="3" t="n"/>
     </row>
@@ -5339,7 +5329,7 @@
         <v>1</v>
       </c>
       <c r="AM50" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN50" s="3" t="n"/>
     </row>
@@ -5432,9 +5422,11 @@
       <c r="AJ51" s="3" t="n"/>
       <c r="AK51" s="3" t="n"/>
       <c r="AL51" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM51" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM51" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN51" s="3" t="n"/>
     </row>
     <row r="52">
@@ -5529,7 +5521,7 @@
         <v>1</v>
       </c>
       <c r="AM52" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN52" s="3" t="n"/>
     </row>
@@ -5719,7 +5711,7 @@
         <v>1</v>
       </c>
       <c r="AM54" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN54" s="3" t="n"/>
     </row>
@@ -5812,9 +5804,11 @@
       <c r="AJ55" s="3" t="n"/>
       <c r="AK55" s="3" t="n"/>
       <c r="AL55" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM55" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM55" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN55" s="3" t="n"/>
     </row>
     <row r="56">
@@ -5906,11 +5900,9 @@
       <c r="AJ56" s="3" t="n"/>
       <c r="AK56" s="3" t="n"/>
       <c r="AL56" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM56" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM56" s="10" t="n"/>
       <c r="AN56" s="3" t="n"/>
     </row>
     <row r="57">
@@ -6002,9 +5994,11 @@
       <c r="AJ57" s="3" t="n"/>
       <c r="AK57" s="3" t="n"/>
       <c r="AL57" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM57" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM57" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN57" s="3" t="n"/>
     </row>
     <row r="58">
@@ -6284,11 +6278,9 @@
       <c r="AJ60" s="3" t="n"/>
       <c r="AK60" s="3" t="n"/>
       <c r="AL60" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM60" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM60" s="10" t="n"/>
       <c r="AN60" s="3" t="n"/>
     </row>
     <row r="61">
@@ -6568,11 +6560,9 @@
       <c r="AJ63" s="3" t="n"/>
       <c r="AK63" s="3" t="n"/>
       <c r="AL63" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM63" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM63" s="10" t="n"/>
       <c r="AN63" s="3" t="n"/>
     </row>
     <row r="64">
@@ -6664,11 +6654,9 @@
       <c r="AJ64" s="3" t="n"/>
       <c r="AK64" s="3" t="n"/>
       <c r="AL64" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM64" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM64" s="10" t="n"/>
       <c r="AN64" s="3" t="n"/>
     </row>
     <row r="65">
@@ -6763,7 +6751,7 @@
         <v>1</v>
       </c>
       <c r="AM65" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN65" s="3" t="n"/>
     </row>
@@ -6859,7 +6847,7 @@
         <v>1</v>
       </c>
       <c r="AM66" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN66" s="3" t="n"/>
     </row>
@@ -7140,11 +7128,9 @@
       <c r="AJ69" s="3" t="n"/>
       <c r="AK69" s="3" t="n"/>
       <c r="AL69" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM69" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM69" s="10" t="n"/>
       <c r="AN69" s="3" t="n"/>
     </row>
     <row r="70">
@@ -7236,11 +7222,9 @@
       <c r="AJ70" s="3" t="n"/>
       <c r="AK70" s="3" t="n"/>
       <c r="AL70" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM70" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM70" s="10" t="n"/>
       <c r="AN70" s="3" t="n"/>
     </row>
     <row r="71">
@@ -7332,9 +7316,11 @@
       <c r="AJ71" s="3" t="n"/>
       <c r="AK71" s="3" t="n"/>
       <c r="AL71" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM71" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM71" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN71" s="3" t="n"/>
     </row>
     <row r="72">
@@ -7520,11 +7506,9 @@
       <c r="AJ73" s="3" t="n"/>
       <c r="AK73" s="3" t="n"/>
       <c r="AL73" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM73" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM73" s="10" t="n"/>
       <c r="AN73" s="3" t="n"/>
     </row>
     <row r="74">
@@ -7616,11 +7600,9 @@
       <c r="AJ74" s="3" t="n"/>
       <c r="AK74" s="3" t="n"/>
       <c r="AL74" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM74" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM74" s="10" t="n"/>
       <c r="AN74" s="3" t="n"/>
     </row>
     <row r="75">
@@ -7712,9 +7694,11 @@
       <c r="AJ75" s="3" t="n"/>
       <c r="AK75" s="3" t="n"/>
       <c r="AL75" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM75" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM75" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN75" s="3" t="n"/>
     </row>
     <row r="76">
@@ -7806,9 +7790,11 @@
       <c r="AJ76" s="3" t="n"/>
       <c r="AK76" s="3" t="n"/>
       <c r="AL76" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM76" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM76" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN76" s="3" t="n"/>
     </row>
     <row r="77">
@@ -8088,9 +8074,11 @@
       <c r="AJ79" s="3" t="n"/>
       <c r="AK79" s="3" t="n"/>
       <c r="AL79" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM79" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM79" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN79" s="3" t="n"/>
     </row>
     <row r="80">
@@ -8185,7 +8173,7 @@
         <v>1</v>
       </c>
       <c r="AM80" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN80" s="3" t="n"/>
     </row>
@@ -8372,9 +8360,11 @@
       <c r="AJ82" s="3" t="n"/>
       <c r="AK82" s="3" t="n"/>
       <c r="AL82" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM82" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM82" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN82" s="3" t="n"/>
     </row>
     <row r="83">
@@ -8469,7 +8459,7 @@
         <v>1</v>
       </c>
       <c r="AM83" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN83" s="3" t="n"/>
     </row>
@@ -8750,9 +8740,11 @@
       <c r="AJ86" s="3" t="n"/>
       <c r="AK86" s="3" t="n"/>
       <c r="AL86" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM86" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM86" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN86" s="3" t="n"/>
     </row>
     <row r="87">
@@ -8941,7 +8933,7 @@
         <v>1</v>
       </c>
       <c r="AM88" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN88" s="3" t="n"/>
     </row>
@@ -9034,11 +9026,9 @@
       <c r="AJ89" s="3" t="n"/>
       <c r="AK89" s="3" t="n"/>
       <c r="AL89" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM89" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM89" s="10" t="n"/>
       <c r="AN89" s="3" t="n"/>
     </row>
     <row r="90">
@@ -9130,11 +9120,9 @@
       <c r="AJ90" s="3" t="n"/>
       <c r="AK90" s="3" t="n"/>
       <c r="AL90" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM90" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM90" s="10" t="n"/>
       <c r="AN90" s="3" t="n"/>
     </row>
     <row r="91">
@@ -9226,11 +9214,9 @@
       <c r="AJ91" s="3" t="n"/>
       <c r="AK91" s="3" t="n"/>
       <c r="AL91" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM91" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM91" s="10" t="n"/>
       <c r="AN91" s="3" t="n"/>
     </row>
     <row r="92">
@@ -9322,9 +9308,11 @@
       <c r="AJ92" s="3" t="n"/>
       <c r="AK92" s="3" t="n"/>
       <c r="AL92" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM92" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM92" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN92" s="3" t="n"/>
     </row>
     <row r="93">
@@ -9513,7 +9501,7 @@
         <v>1</v>
       </c>
       <c r="AM94" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN94" s="3" t="n"/>
     </row>
@@ -9700,9 +9688,11 @@
       <c r="AJ96" s="3" t="n"/>
       <c r="AK96" s="3" t="n"/>
       <c r="AL96" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM96" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM96" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN96" s="3" t="n"/>
     </row>
     <row r="97">
@@ -10079,7 +10069,7 @@
         <v>1</v>
       </c>
       <c r="AM100" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN100" s="3" t="n"/>
     </row>
@@ -10172,9 +10162,11 @@
       <c r="AJ101" s="3" t="n"/>
       <c r="AK101" s="3" t="n"/>
       <c r="AL101" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM101" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM101" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN101" s="3" t="n"/>
     </row>
     <row r="102">
@@ -10269,7 +10261,7 @@
         <v>1</v>
       </c>
       <c r="AM102" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN102" s="3" t="n"/>
     </row>
@@ -10456,9 +10448,11 @@
       <c r="AJ104" s="3" t="n"/>
       <c r="AK104" s="3" t="n"/>
       <c r="AL104" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM104" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM104" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN104" s="3" t="n"/>
     </row>
     <row r="105">
@@ -10550,9 +10544,11 @@
       <c r="AJ105" s="3" t="n"/>
       <c r="AK105" s="3" t="n"/>
       <c r="AL105" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM105" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM105" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN105" s="3" t="n"/>
     </row>
     <row r="106">
@@ -10644,9 +10640,11 @@
       <c r="AJ106" s="3" t="n"/>
       <c r="AK106" s="3" t="n"/>
       <c r="AL106" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM106" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM106" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN106" s="3" t="n"/>
     </row>
     <row r="107">
@@ -10738,9 +10736,11 @@
       <c r="AJ107" s="3" t="n"/>
       <c r="AK107" s="3" t="n"/>
       <c r="AL107" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM107" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM107" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN107" s="3" t="n"/>
     </row>
     <row r="108">
@@ -10832,9 +10832,11 @@
       <c r="AJ108" s="3" t="n"/>
       <c r="AK108" s="3" t="n"/>
       <c r="AL108" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM108" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM108" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN108" s="3" t="n"/>
     </row>
     <row r="109">
@@ -10929,7 +10931,7 @@
         <v>1</v>
       </c>
       <c r="AM109" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN109" s="3" t="n"/>
     </row>
@@ -11116,9 +11118,11 @@
       <c r="AJ111" s="3" t="n"/>
       <c r="AK111" s="3" t="n"/>
       <c r="AL111" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM111" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM111" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN111" s="3" t="n"/>
     </row>
     <row r="112">
@@ -11210,9 +11214,11 @@
       <c r="AJ112" s="3" t="n"/>
       <c r="AK112" s="3" t="n"/>
       <c r="AL112" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM112" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM112" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN112" s="3" t="n"/>
     </row>
     <row r="113">
@@ -11304,11 +11310,9 @@
       <c r="AJ113" s="3" t="n"/>
       <c r="AK113" s="3" t="n"/>
       <c r="AL113" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM113" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM113" s="10" t="n"/>
       <c r="AN113" s="3" t="n"/>
     </row>
     <row r="114">
@@ -11400,9 +11404,11 @@
       <c r="AJ114" s="3" t="n"/>
       <c r="AK114" s="3" t="n"/>
       <c r="AL114" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM114" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM114" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN114" s="3" t="n"/>
     </row>
     <row r="115">
@@ -11497,7 +11503,7 @@
         <v>1</v>
       </c>
       <c r="AM115" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN115" s="3" t="n"/>
     </row>
@@ -11684,9 +11690,11 @@
       <c r="AJ117" s="3" t="n"/>
       <c r="AK117" s="3" t="n"/>
       <c r="AL117" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM117" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM117" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN117" s="3" t="n"/>
     </row>
     <row r="118">
@@ -11875,7 +11883,7 @@
         <v>1</v>
       </c>
       <c r="AM119" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN119" s="3" t="n"/>
     </row>
@@ -11968,9 +11976,11 @@
       <c r="AJ120" s="3" t="n"/>
       <c r="AK120" s="3" t="n"/>
       <c r="AL120" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM120" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM120" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN120" s="3" t="n"/>
     </row>
     <row r="121">
@@ -12062,11 +12072,9 @@
       <c r="AJ121" s="3" t="n"/>
       <c r="AK121" s="3" t="n"/>
       <c r="AL121" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM121" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM121" s="10" t="n"/>
       <c r="AN121" s="3" t="n"/>
     </row>
     <row r="122">
@@ -12158,11 +12166,9 @@
       <c r="AJ122" s="3" t="n"/>
       <c r="AK122" s="3" t="n"/>
       <c r="AL122" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM122" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM122" s="10" t="n"/>
       <c r="AN122" s="3" t="n"/>
     </row>
     <row r="123">
@@ -12254,11 +12260,9 @@
       <c r="AJ123" s="3" t="n"/>
       <c r="AK123" s="3" t="n"/>
       <c r="AL123" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM123" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM123" s="10" t="n"/>
       <c r="AN123" s="3" t="n"/>
     </row>
     <row r="124">
@@ -12350,11 +12354,9 @@
       <c r="AJ124" s="3" t="n"/>
       <c r="AK124" s="3" t="n"/>
       <c r="AL124" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM124" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM124" s="10" t="n"/>
       <c r="AN124" s="3" t="n"/>
     </row>
     <row r="125">
@@ -12446,9 +12448,11 @@
       <c r="AJ125" s="3" t="n"/>
       <c r="AK125" s="3" t="n"/>
       <c r="AL125" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM125" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM125" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN125" s="3" t="n"/>
     </row>
     <row r="126">
@@ -12543,7 +12547,7 @@
         <v>1</v>
       </c>
       <c r="AM126" s="10" t="n">
-        <v>46217.4577819237</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN126" s="3" t="n"/>
     </row>
@@ -12636,9 +12640,11 @@
       <c r="AJ127" s="3" t="n"/>
       <c r="AK127" s="3" t="n"/>
       <c r="AL127" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM127" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM127" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN127" s="3" t="n"/>
     </row>
     <row r="128">
@@ -12730,9 +12736,11 @@
       <c r="AJ128" s="3" t="n"/>
       <c r="AK128" s="3" t="n"/>
       <c r="AL128" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM128" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM128" s="10" t="n">
+        <v>46217.62198509788</v>
+      </c>
       <c r="AN128" s="3" t="n"/>
     </row>
     <row r="129">
@@ -12824,9 +12832,11 @@
       <c r="AJ129" s="3" t="n"/>
       <c r="AK129" s="3" t="n"/>
       <c r="AL129" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM129" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM129" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN129" s="3" t="n"/>
     </row>
     <row r="130">
@@ -12918,11 +12928,9 @@
       <c r="AJ130" s="3" t="n"/>
       <c r="AK130" s="3" t="n"/>
       <c r="AL130" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM130" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM130" s="10" t="n"/>
       <c r="AN130" s="3" t="n"/>
     </row>
     <row r="131">
@@ -13108,11 +13116,9 @@
       <c r="AJ132" s="3" t="n"/>
       <c r="AK132" s="3" t="n"/>
       <c r="AL132" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM132" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM132" s="10" t="n"/>
       <c r="AN132" s="3" t="n"/>
     </row>
     <row r="133">
@@ -13204,11 +13210,9 @@
       <c r="AJ133" s="3" t="n"/>
       <c r="AK133" s="3" t="n"/>
       <c r="AL133" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM133" s="10" t="n">
-        <v>46217.4577819237</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM133" s="10" t="n"/>
       <c r="AN133" s="3" t="n"/>
     </row>
     <row r="134">
@@ -13300,9 +13304,11 @@
       <c r="AJ134" s="3" t="n"/>
       <c r="AK134" s="3" t="n"/>
       <c r="AL134" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM134" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM134" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN134" s="3" t="n"/>
     </row>
     <row r="135">
@@ -13394,9 +13400,11 @@
       <c r="AJ135" s="3" t="n"/>
       <c r="AK135" s="3" t="n"/>
       <c r="AL135" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM135" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM135" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN135" s="3" t="n"/>
     </row>
     <row r="136">
@@ -13585,7 +13593,7 @@
         <v>1</v>
       </c>
       <c r="AM137" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN137" s="3" t="n"/>
     </row>
@@ -13681,7 +13689,7 @@
         <v>1</v>
       </c>
       <c r="AM138" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198509788</v>
       </c>
       <c r="AN138" s="3" t="n"/>
     </row>
@@ -13774,11 +13782,9 @@
       <c r="AJ139" s="3" t="n"/>
       <c r="AK139" s="3" t="n"/>
       <c r="AL139" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM139" s="10" t="n">
-        <v>46217.45778064815</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM139" s="10" t="n"/>
       <c r="AN139" s="3" t="n"/>
     </row>
     <row r="140">
@@ -13964,9 +13970,11 @@
       <c r="AJ141" s="3" t="n"/>
       <c r="AK141" s="3" t="n"/>
       <c r="AL141" s="3" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM141" s="10" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="AM141" s="10" t="n">
+        <v>46217.62198391204</v>
+      </c>
       <c r="AN141" s="3" t="n"/>
     </row>
     <row r="142">
@@ -14061,7 +14069,7 @@
         <v>1</v>
       </c>
       <c r="AM142" s="10" t="n">
-        <v>46217.45778210896</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN142" s="3" t="n"/>
     </row>
@@ -14345,7 +14353,7 @@
         <v>1</v>
       </c>
       <c r="AM145" s="10" t="n">
-        <v>46217.45778210896</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN145" s="3" t="n"/>
     </row>
@@ -14438,11 +14446,9 @@
       <c r="AJ146" s="3" t="n"/>
       <c r="AK146" s="3" t="n"/>
       <c r="AL146" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM146" s="10" t="n">
-        <v>46217.45778210896</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AM146" s="10" t="n"/>
       <c r="AN146" s="3" t="n"/>
     </row>
     <row r="147">
@@ -14537,7 +14543,7 @@
         <v>1</v>
       </c>
       <c r="AM147" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN147" s="3" t="n"/>
     </row>
@@ -14633,7 +14639,7 @@
         <v>1</v>
       </c>
       <c r="AM148" s="10" t="n">
-        <v>46217.45778064815</v>
+        <v>46217.62198391204</v>
       </c>
       <c r="AN148" s="3" t="n"/>
     </row>

</xml_diff>